<commit_message>
Excels: valores calculados en cache (se ven en cualquier visor) + fix d en losa (usaba area en vez de diametro)
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/DISENO-LOSA-NERVADA-1D.xlsx
+++ b/Proyectos/Diseno-Estructural/DISENO-LOSA-NERVADA-1D.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Geometria y Verificaciones" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Predimensionamiento" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Avaluo de Cargas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Nervios Entrepiso" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Nervios Cubierta" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Loseta" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Deflexiones" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geometria y Verificaciones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Predimensionamiento" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avaluo de Cargas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nervios Entrepiso" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nervios Cubierta" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loseta" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deflexiones" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -721,7 +721,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>  </t>
+          <t xml:space="preserve">  </t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="B16" s="12">
         <f>B10-B7</f>
-        <v/>
+        <v>0.65</v>
       </c>
     </row>
     <row r="17">
@@ -899,7 +899,7 @@
       </c>
       <c r="B17" s="12">
         <f>B8-B9</f>
-        <v/>
+        <v>0.28</v>
       </c>
     </row>
     <row r="18">
@@ -909,8 +909,8 @@
         </is>
       </c>
       <c r="B18" s="13">
-        <f>B8*1000-B11*1000-B13/2</f>
-        <v/>
+        <f>B8*1000-B11*1000-B12/2</f>
+        <v>303.65</v>
       </c>
     </row>
     <row r="19">
@@ -921,7 +921,7 @@
       </c>
       <c r="B19" s="14">
         <f>B8/B7</f>
-        <v/>
+        <v>2.266666667</v>
       </c>
     </row>
     <row r="21">
@@ -961,16 +961,16 @@
       </c>
       <c r="B23" s="16">
         <f>B7*1000</f>
-        <v/>
+        <v>150</v>
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="17" t="str">
         <f>IF(B7*1000&gt;=100,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="24">
@@ -981,16 +981,16 @@
       </c>
       <c r="B24" s="16">
         <f>B19</f>
-        <v/>
+        <v>2.266666667</v>
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="D24" s="17">
+      <c r="D24" s="17" t="str">
         <f>IF(B19&lt;=3.5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="25">
@@ -1001,16 +1001,16 @@
       </c>
       <c r="B25" s="16">
         <f>B16*1000</f>
-        <v/>
+        <v>650</v>
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
           <t>750</t>
         </is>
       </c>
-      <c r="D25" s="17">
+      <c r="D25" s="17" t="str">
         <f>IF(B16*1000&lt;=750,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="26">
@@ -1021,15 +1021,15 @@
       </c>
       <c r="B26" s="16">
         <f>B9*1000</f>
-        <v/>
+        <v>60</v>
       </c>
       <c r="C26" s="16">
         <f>B16*1000/12</f>
-        <v/>
-      </c>
-      <c r="D26" s="17">
+        <v>54.16666667</v>
+      </c>
+      <c r="D26" s="17" t="str">
         <f>IF(B9*1000&gt;=B16*1000/12,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="27">
@@ -1040,16 +1040,16 @@
       </c>
       <c r="B27" s="16">
         <f>B9*1000</f>
-        <v/>
+        <v>60</v>
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="D27" s="17">
+      <c r="D27" s="17" t="str">
         <f>IF(B9*1000&gt;=45,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="29">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="B4" s="14">
         <f>'Geometria y Verificaciones'!B8</f>
-        <v/>
+        <v>0.34</v>
       </c>
     </row>
     <row r="6">
@@ -1163,15 +1163,15 @@
       </c>
       <c r="E7" s="22">
         <f>B7/D7</f>
-        <v/>
+        <v>0.1189189189</v>
       </c>
       <c r="F7" s="23">
         <f>$B$4</f>
-        <v/>
-      </c>
-      <c r="G7" s="17">
+        <v>0.34</v>
+      </c>
+      <c r="G7" s="17" t="str">
         <f>IF(F7&gt;=E7,"CUMPLE","AUMENTAR h")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="8">
@@ -1193,15 +1193,15 @@
       </c>
       <c r="E8" s="22">
         <f>B8/D8</f>
-        <v/>
+        <v>0.1945945946</v>
       </c>
       <c r="F8" s="23">
         <f>$B$4</f>
-        <v/>
-      </c>
-      <c r="G8" s="17">
+        <v>0.34</v>
+      </c>
+      <c r="G8" s="17" t="str">
         <f>IF(F8&gt;=E8,"CUMPLE","AUMENTAR h")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="9">
@@ -1223,15 +1223,15 @@
       </c>
       <c r="E9" s="22">
         <f>B9/D9</f>
-        <v/>
+        <v>0.2594594595</v>
       </c>
       <c r="F9" s="23">
         <f>$B$4</f>
-        <v/>
-      </c>
-      <c r="G9" s="17">
+        <v>0.34</v>
+      </c>
+      <c r="G9" s="17" t="str">
         <f>IF(F9&gt;=E9,"CUMPLE","AUMENTAR h")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="10">
@@ -1253,15 +1253,15 @@
       </c>
       <c r="E10" s="22">
         <f>B10/D10</f>
-        <v/>
+        <v>0.2783783784</v>
       </c>
       <c r="F10" s="23">
         <f>$B$4</f>
-        <v/>
-      </c>
-      <c r="G10" s="17">
+        <v>0.34</v>
+      </c>
+      <c r="G10" s="17" t="str">
         <f>IF(F10&gt;=E10,"CUMPLE","AUMENTAR h")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="12">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="B5" s="12">
         <f>'Geometria y Verificaciones'!B6*'Geometria y Verificaciones'!B9</f>
-        <v/>
+        <v>1.44</v>
       </c>
     </row>
     <row r="6">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B6" s="12">
         <f>'Geometria y Verificaciones'!B6*'Geometria y Verificaciones'!B7*('Geometria y Verificaciones'!B8-'Geometria y Verificaciones'!B9)/'Geometria y Verificaciones'!B10</f>
-        <v/>
+        <v>1.26</v>
       </c>
     </row>
     <row r="7">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="B8" s="12">
         <f>SUM(B5:B7)</f>
-        <v/>
+        <v>3.05</v>
       </c>
     </row>
     <row r="10">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="B14" s="12">
         <f>B8+SUM(B11:B13)</f>
-        <v/>
+        <v>7.04</v>
       </c>
     </row>
     <row r="15">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B16" s="12">
         <f>1.2*B14+1.6*B15</f>
-        <v/>
+        <v>11.328</v>
       </c>
     </row>
     <row r="18">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="B21" s="12">
         <f>B8+SUM(B19:B20)</f>
-        <v/>
+        <v>4.376</v>
       </c>
     </row>
     <row r="22">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="B23" s="12">
         <f>1.2*B21+1.6*B22</f>
-        <v/>
+        <v>13.2512</v>
       </c>
     </row>
     <row r="25">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B5" s="25">
         <f>'Geometria y Verificaciones'!B4</f>
-        <v/>
+        <v>28</v>
       </c>
     </row>
     <row r="6">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="B6" s="25">
         <f>'Geometria y Verificaciones'!B5</f>
-        <v/>
+        <v>420</v>
       </c>
     </row>
     <row r="7">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="B7" s="25">
         <f>'Geometria y Verificaciones'!B7*1000</f>
-        <v/>
+        <v>150</v>
       </c>
     </row>
     <row r="8">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="B8" s="25">
         <f>'Geometria y Verificaciones'!B8</f>
-        <v/>
+        <v>0.34</v>
       </c>
     </row>
     <row r="9">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="B9" s="25">
         <f>'Geometria y Verificaciones'!B9*1000</f>
-        <v/>
+        <v>60</v>
       </c>
     </row>
     <row r="10">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" s="25">
         <f>'Geometria y Verificaciones'!B10</f>
-        <v/>
+        <v>0.8</v>
       </c>
     </row>
     <row r="11">
@@ -1624,8 +1624,8 @@
         </is>
       </c>
       <c r="B11" s="25">
-        <f>'Geometria y Verificaciones'!B8*1000-'Geometria y Verificaciones'!B11*1000-'Geometria y Verificaciones'!B13/2</f>
-        <v/>
+        <f>'Geometria y Verificaciones'!B8*1000-'Geometria y Verificaciones'!B11*1000-'Geometria y Verificaciones'!B12/2</f>
+        <v>303.65</v>
       </c>
     </row>
     <row r="12">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="B12" s="25">
         <f>'Geometria y Verificaciones'!B13</f>
-        <v/>
+        <v>129</v>
       </c>
     </row>
     <row r="13">
@@ -1646,8 +1646,8 @@
         </is>
       </c>
       <c r="B13" s="25">
-        <f>MAX(0.25*SQRT('Geometria y Verificaciones'!B4)/'Geometria y Verificaciones'!B5,1.4/'Geometria y Verificaciones'!B5)*'Geometria y Verificaciones'!B7*1000*('Geometria y Verificaciones'!B8*1000-'Geometria y Verificaciones'!B11*1000-'Geometria y Verificaciones'!B13/2)</f>
-        <v/>
+        <f>MAX(0.25*SQRT('Geometria y Verificaciones'!B4)/'Geometria y Verificaciones'!B5,1.4/'Geometria y Verificaciones'!B5)*'Geometria y Verificaciones'!B7*1000*('Geometria y Verificaciones'!B8*1000-'Geometria y Verificaciones'!B11*1000-'Geometria y Verificaciones'!B12/2)</f>
+        <v>151.825</v>
       </c>
     </row>
     <row r="14">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="B14" s="25">
         <f>'Avaluo de Cargas'!B16</f>
-        <v/>
+        <v>11.328</v>
       </c>
     </row>
     <row r="15">
@@ -1841,91 +1841,91 @@
       </c>
       <c r="C19" s="23">
         <f>B19-$B$15</f>
-        <v/>
+        <v>1.85</v>
       </c>
       <c r="D19" s="27">
         <f>MIN(C19*1000/4,$B$7+16*$B$9,$B$10*1000)</f>
-        <v/>
+        <v>462.5</v>
       </c>
       <c r="E19" s="23">
         <f>$B$14*$B$10</f>
-        <v/>
+        <v>9.0624</v>
       </c>
       <c r="F19" s="16">
         <f>E19*C19^2/10</f>
-        <v/>
+        <v>3.1016064</v>
       </c>
       <c r="G19" s="16">
         <f>E19*C19^2/14</f>
-        <v/>
+        <v>2.215433143</v>
       </c>
       <c r="H19" s="16">
         <f>1.15*E19*C19/2</f>
-        <v/>
+        <v>9.640128</v>
       </c>
       <c r="I19" s="22">
         <f>G19*1000000/(0.9*D19*$B$11^2)</f>
-        <v/>
+        <v>0.05772418781</v>
       </c>
       <c r="J19" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*I19/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.0001376056186</v>
       </c>
       <c r="K19" s="27">
         <f>J19*D19*$B$11</f>
-        <v/>
+        <v>19.32507507</v>
       </c>
       <c r="L19" s="16">
         <f>N19*$B$6/(0.85*$B$5*D19)</f>
-        <v/>
-      </c>
-      <c r="M19" s="17">
+        <v>5.793004769</v>
+      </c>
+      <c r="M19" s="17" t="str">
         <f>IF(L19&lt;=$B$9,"Si (T)","revisar")</f>
-        <v/>
+        <v>Si (T)</v>
       </c>
       <c r="N19" s="27">
         <f>MAX(K19,$B$13)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="O19" s="29">
         <f>ROUNDUP(N19/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="P19" s="22">
         <f>F19*1000000/(0.9*$B$7*$B$11^2)</f>
-        <v/>
+        <v>0.2491760774</v>
       </c>
       <c r="Q19" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*P19/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.0005964149999</v>
       </c>
       <c r="R19" s="27">
         <f>Q19*$B$7*$B$11</f>
-        <v/>
+        <v>27.16521221</v>
       </c>
       <c r="S19" s="27">
         <f>MAX(R19,$B$13)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="T19" s="29">
         <f>ROUNDUP(S19/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="U19" s="16">
         <f>0.17*SQRT($B$5)*$B$7*$B$11/1000</f>
-        <v/>
+        <v>40.97250167</v>
       </c>
       <c r="V19" s="16">
         <f>0.75*1.1*U19</f>
-        <v/>
-      </c>
-      <c r="W19" s="17">
+        <v>33.80231387</v>
+      </c>
+      <c r="W19" s="17" t="str">
         <f>IF(H19&lt;=V19,"No requiere","Requiere")</f>
-        <v/>
-      </c>
-      <c r="X19" s="17">
+        <v>No requiere</v>
+      </c>
+      <c r="X19" s="17" t="str">
         <f>IF($B$8&gt;=C19/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="20">
@@ -1939,91 +1939,91 @@
       </c>
       <c r="C20" s="23">
         <f>B20-$B$15</f>
-        <v/>
+        <v>3.25</v>
       </c>
       <c r="D20" s="27">
         <f>MIN(C20*1000/4,$B$7+16*$B$9,$B$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="E20" s="23">
         <f>$B$14*$B$10</f>
-        <v/>
+        <v>9.0624</v>
       </c>
       <c r="F20" s="16">
         <f>E20*C20^2/10</f>
-        <v/>
+        <v>9.57216</v>
       </c>
       <c r="G20" s="16">
         <f>E20*C20^2/14</f>
-        <v/>
+        <v>6.837257143</v>
       </c>
       <c r="H20" s="16">
         <f>1.15*E20*C20/2</f>
-        <v/>
+        <v>16.93536</v>
       </c>
       <c r="I20" s="22">
         <f>G20*1000000/(0.9*D20*$B$11^2)</f>
-        <v/>
+        <v>0.1029918469</v>
       </c>
       <c r="J20" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*I20/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.0002457515699</v>
       </c>
       <c r="K20" s="27">
         <f>J20*D20*$B$11</f>
-        <v/>
+        <v>59.69797136</v>
       </c>
       <c r="L20" s="16">
         <f>N20*$B$6/(0.85*$B$5*D20)</f>
-        <v/>
-      </c>
-      <c r="M20" s="17">
+        <v>3.349080882</v>
+      </c>
+      <c r="M20" s="17" t="str">
         <f>IF(L20&lt;=$B$9,"Si (T)","revisar")</f>
-        <v/>
+        <v>Si (T)</v>
       </c>
       <c r="N20" s="27">
         <f>MAX(K20,$B$13)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="O20" s="29">
         <f>ROUNDUP(N20/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="P20" s="22">
         <f>F20*1000000/(0.9*$B$7*$B$11^2)</f>
-        <v/>
+        <v>0.7690057903</v>
       </c>
       <c r="Q20" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*P20/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.001861542708</v>
       </c>
       <c r="R20" s="27">
         <f>Q20*$B$7*$B$11</f>
-        <v/>
+        <v>84.78861649</v>
       </c>
       <c r="S20" s="27">
         <f>MAX(R20,$B$13)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="T20" s="29">
         <f>ROUNDUP(S20/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="U20" s="16">
         <f>0.17*SQRT($B$5)*$B$7*$B$11/1000</f>
-        <v/>
+        <v>40.97250167</v>
       </c>
       <c r="V20" s="16">
         <f>0.75*1.1*U20</f>
-        <v/>
-      </c>
-      <c r="W20" s="17">
+        <v>33.80231387</v>
+      </c>
+      <c r="W20" s="17" t="str">
         <f>IF(H20&lt;=V20,"No requiere","Requiere")</f>
-        <v/>
-      </c>
-      <c r="X20" s="17">
+        <v>No requiere</v>
+      </c>
+      <c r="X20" s="17" t="str">
         <f>IF($B$8&gt;=C20/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="21">
@@ -2037,91 +2037,91 @@
       </c>
       <c r="C21" s="23">
         <f>B21-$B$15</f>
-        <v/>
+        <v>4.45</v>
       </c>
       <c r="D21" s="27">
         <f>MIN(C21*1000/4,$B$7+16*$B$9,$B$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="E21" s="23">
         <f>$B$14*$B$10</f>
-        <v/>
+        <v>9.0624</v>
       </c>
       <c r="F21" s="16">
         <f>E21*C21^2/10</f>
-        <v/>
+        <v>17.9458176</v>
       </c>
       <c r="G21" s="16">
         <f>E21*C21^2/14</f>
-        <v/>
+        <v>12.81844114</v>
       </c>
       <c r="H21" s="16">
         <f>1.15*E21*C21/2</f>
-        <v/>
+        <v>23.188416</v>
       </c>
       <c r="I21" s="22">
         <f>G21*1000000/(0.9*D21*$B$11^2)</f>
-        <v/>
+        <v>0.1930883833</v>
       </c>
       <c r="J21" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*I21/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.0004616144332</v>
       </c>
       <c r="K21" s="27">
         <f>J21*D21*$B$11</f>
-        <v/>
+        <v>112.1353781</v>
       </c>
       <c r="L21" s="16">
         <f>N21*$B$6/(0.85*$B$5*D21)</f>
-        <v/>
-      </c>
-      <c r="M21" s="17">
+        <v>3.349080882</v>
+      </c>
+      <c r="M21" s="17" t="str">
         <f>IF(L21&lt;=$B$9,"Si (T)","revisar")</f>
-        <v/>
+        <v>Si (T)</v>
       </c>
       <c r="N21" s="27">
         <f>MAX(K21,$B$13)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="O21" s="29">
         <f>ROUNDUP(N21/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="P21" s="22">
         <f>F21*1000000/(0.9*$B$7*$B$11^2)</f>
-        <v/>
+        <v>1.441726595</v>
       </c>
       <c r="Q21" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*P21/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.003543472336</v>
       </c>
       <c r="R21" s="27">
         <f>Q21*$B$7*$B$11</f>
-        <v/>
+        <v>161.3963062</v>
       </c>
       <c r="S21" s="27">
         <f>MAX(R21,$B$13)</f>
-        <v/>
+        <v>161.3963062</v>
       </c>
       <c r="T21" s="29">
         <f>ROUNDUP(S21/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="U21" s="16">
         <f>0.17*SQRT($B$5)*$B$7*$B$11/1000</f>
-        <v/>
+        <v>40.97250167</v>
       </c>
       <c r="V21" s="16">
         <f>0.75*1.1*U21</f>
-        <v/>
-      </c>
-      <c r="W21" s="17">
+        <v>33.80231387</v>
+      </c>
+      <c r="W21" s="17" t="str">
         <f>IF(H21&lt;=V21,"No requiere","Requiere")</f>
-        <v/>
-      </c>
-      <c r="X21" s="17">
+        <v>No requiere</v>
+      </c>
+      <c r="X21" s="17" t="str">
         <f>IF($B$8&gt;=C21/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="22">
@@ -2135,91 +2135,91 @@
       </c>
       <c r="C22" s="23">
         <f>B22-$B$15</f>
-        <v/>
+        <v>4.8</v>
       </c>
       <c r="D22" s="27">
         <f>MIN(C22*1000/4,$B$7+16*$B$9,$B$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="E22" s="23">
         <f>$B$14*$B$10</f>
-        <v/>
+        <v>9.0624</v>
       </c>
       <c r="F22" s="16">
         <f>E22*C22^2/10</f>
-        <v/>
+        <v>20.8797696</v>
       </c>
       <c r="G22" s="16">
         <f>E22*C22^2/14</f>
-        <v/>
+        <v>14.91412114</v>
       </c>
       <c r="H22" s="16">
         <f>1.15*E22*C22/2</f>
-        <v/>
+        <v>25.012224</v>
       </c>
       <c r="I22" s="22">
         <f>G22*1000000/(0.9*D22*$B$11^2)</f>
-        <v/>
+        <v>0.2246562985</v>
       </c>
       <c r="J22" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*I22/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.0005374445961</v>
       </c>
       <c r="K22" s="27">
         <f>J22*D22*$B$11</f>
-        <v/>
+        <v>130.5560413</v>
       </c>
       <c r="L22" s="16">
         <f>N22*$B$6/(0.85*$B$5*D22)</f>
-        <v/>
-      </c>
-      <c r="M22" s="17">
+        <v>3.349080882</v>
+      </c>
+      <c r="M22" s="17" t="str">
         <f>IF(L22&lt;=$B$9,"Si (T)","revisar")</f>
-        <v/>
+        <v>Si (T)</v>
       </c>
       <c r="N22" s="27">
         <f>MAX(K22,$B$13)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="O22" s="29">
         <f>ROUNDUP(N22/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="P22" s="22">
         <f>F22*1000000/(0.9*$B$7*$B$11^2)</f>
-        <v/>
+        <v>1.677433696</v>
       </c>
       <c r="Q22" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*P22/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.00414552547</v>
       </c>
       <c r="R22" s="27">
         <f>Q22*$B$7*$B$11</f>
-        <v/>
+        <v>188.8183213</v>
       </c>
       <c r="S22" s="27">
         <f>MAX(R22,$B$13)</f>
-        <v/>
+        <v>188.8183213</v>
       </c>
       <c r="T22" s="29">
         <f>ROUNDUP(S22/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="U22" s="16">
         <f>0.17*SQRT($B$5)*$B$7*$B$11/1000</f>
-        <v/>
+        <v>40.97250167</v>
       </c>
       <c r="V22" s="16">
         <f>0.75*1.1*U22</f>
-        <v/>
-      </c>
-      <c r="W22" s="17">
+        <v>33.80231387</v>
+      </c>
+      <c r="W22" s="17" t="str">
         <f>IF(H22&lt;=V22,"No requiere","Requiere")</f>
-        <v/>
-      </c>
-      <c r="X22" s="17">
+        <v>No requiere</v>
+      </c>
+      <c r="X22" s="17" t="str">
         <f>IF($B$8&gt;=C22/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="24">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="B5" s="25">
         <f>'Geometria y Verificaciones'!B4</f>
-        <v/>
+        <v>28</v>
       </c>
     </row>
     <row r="6">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="B6" s="25">
         <f>'Geometria y Verificaciones'!B5</f>
-        <v/>
+        <v>420</v>
       </c>
     </row>
     <row r="7">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="B7" s="25">
         <f>'Geometria y Verificaciones'!B7*1000</f>
-        <v/>
+        <v>150</v>
       </c>
     </row>
     <row r="8">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="B8" s="25">
         <f>'Geometria y Verificaciones'!B8</f>
-        <v/>
+        <v>0.34</v>
       </c>
     </row>
     <row r="9">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="B9" s="25">
         <f>'Geometria y Verificaciones'!B9*1000</f>
-        <v/>
+        <v>60</v>
       </c>
     </row>
     <row r="10">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="B10" s="25">
         <f>'Geometria y Verificaciones'!B10</f>
-        <v/>
+        <v>0.8</v>
       </c>
     </row>
     <row r="11">
@@ -2372,8 +2372,8 @@
         </is>
       </c>
       <c r="B11" s="25">
-        <f>'Geometria y Verificaciones'!B8*1000-'Geometria y Verificaciones'!B11*1000-'Geometria y Verificaciones'!B13/2</f>
-        <v/>
+        <f>'Geometria y Verificaciones'!B8*1000-'Geometria y Verificaciones'!B11*1000-'Geometria y Verificaciones'!B12/2</f>
+        <v>303.65</v>
       </c>
     </row>
     <row r="12">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="B12" s="25">
         <f>'Geometria y Verificaciones'!B13</f>
-        <v/>
+        <v>129</v>
       </c>
     </row>
     <row r="13">
@@ -2394,8 +2394,8 @@
         </is>
       </c>
       <c r="B13" s="25">
-        <f>MAX(0.25*SQRT('Geometria y Verificaciones'!B4)/'Geometria y Verificaciones'!B5,1.4/'Geometria y Verificaciones'!B5)*'Geometria y Verificaciones'!B7*1000*('Geometria y Verificaciones'!B8*1000-'Geometria y Verificaciones'!B11*1000-'Geometria y Verificaciones'!B13/2)</f>
-        <v/>
+        <f>MAX(0.25*SQRT('Geometria y Verificaciones'!B4)/'Geometria y Verificaciones'!B5,1.4/'Geometria y Verificaciones'!B5)*'Geometria y Verificaciones'!B7*1000*('Geometria y Verificaciones'!B8*1000-'Geometria y Verificaciones'!B11*1000-'Geometria y Verificaciones'!B12/2)</f>
+        <v>151.825</v>
       </c>
     </row>
     <row r="14">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B14" s="25">
         <f>'Avaluo de Cargas'!B23</f>
-        <v/>
+        <v>13.2512</v>
       </c>
     </row>
     <row r="15">
@@ -2589,91 +2589,91 @@
       </c>
       <c r="C19" s="23">
         <f>B19-$B$15</f>
-        <v/>
+        <v>1.85</v>
       </c>
       <c r="D19" s="27">
         <f>MIN(C19*1000/4,$B$7+16*$B$9,$B$10*1000)</f>
-        <v/>
+        <v>462.5</v>
       </c>
       <c r="E19" s="23">
         <f>$B$14*$B$10</f>
-        <v/>
+        <v>10.60096</v>
       </c>
       <c r="F19" s="16">
         <f>E19*C19^2/10</f>
-        <v/>
+        <v>3.62817856</v>
       </c>
       <c r="G19" s="16">
         <f>E19*C19^2/14</f>
-        <v/>
+        <v>2.591556114</v>
       </c>
       <c r="H19" s="16">
         <f>1.15*E19*C19/2</f>
-        <v/>
+        <v>11.2767712</v>
       </c>
       <c r="I19" s="22">
         <f>G19*1000000/(0.9*D19*$B$11^2)</f>
-        <v/>
+        <v>0.06752425472</v>
       </c>
       <c r="J19" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*I19/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.0001610007519</v>
       </c>
       <c r="K19" s="27">
         <f>J19*D19*$B$11</f>
-        <v/>
+        <v>22.61064372</v>
       </c>
       <c r="L19" s="16">
         <f>N19*$B$6/(0.85*$B$5*D19)</f>
-        <v/>
-      </c>
-      <c r="M19" s="17">
+        <v>5.793004769</v>
+      </c>
+      <c r="M19" s="17" t="str">
         <f>IF(L19&lt;=$B$9,"Si (T)","revisar")</f>
-        <v/>
+        <v>Si (T)</v>
       </c>
       <c r="N19" s="27">
         <f>MAX(K19,$B$13)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="O19" s="29">
         <f>ROUNDUP(N19/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="P19" s="22">
         <f>F19*1000000/(0.9*$B$7*$B$11^2)</f>
-        <v/>
+        <v>0.2914796996</v>
       </c>
       <c r="Q19" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*P19/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.0006983018625</v>
       </c>
       <c r="R19" s="27">
         <f>Q19*$B$7*$B$11</f>
-        <v/>
+        <v>31.80590408</v>
       </c>
       <c r="S19" s="27">
         <f>MAX(R19,$B$13)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="T19" s="29">
         <f>ROUNDUP(S19/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="U19" s="16">
         <f>0.17*SQRT($B$5)*$B$7*$B$11/1000</f>
-        <v/>
+        <v>40.97250167</v>
       </c>
       <c r="V19" s="16">
         <f>0.75*1.1*U19</f>
-        <v/>
-      </c>
-      <c r="W19" s="17">
+        <v>33.80231387</v>
+      </c>
+      <c r="W19" s="17" t="str">
         <f>IF(H19&lt;=V19,"No requiere","Requiere")</f>
-        <v/>
-      </c>
-      <c r="X19" s="17">
+        <v>No requiere</v>
+      </c>
+      <c r="X19" s="17" t="str">
         <f>IF($B$8&gt;=C19/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="20">
@@ -2687,91 +2687,91 @@
       </c>
       <c r="C20" s="23">
         <f>B20-$B$15</f>
-        <v/>
+        <v>3.25</v>
       </c>
       <c r="D20" s="27">
         <f>MIN(C20*1000/4,$B$7+16*$B$9,$B$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="E20" s="23">
         <f>$B$14*$B$10</f>
-        <v/>
+        <v>10.60096</v>
       </c>
       <c r="F20" s="16">
         <f>E20*C20^2/10</f>
-        <v/>
+        <v>11.197264</v>
       </c>
       <c r="G20" s="16">
         <f>E20*C20^2/14</f>
-        <v/>
+        <v>7.998045714</v>
       </c>
       <c r="H20" s="16">
         <f>1.15*E20*C20/2</f>
-        <v/>
+        <v>19.810544</v>
       </c>
       <c r="I20" s="22">
         <f>G20*1000000/(0.9*D20*$B$11^2)</f>
-        <v/>
+        <v>0.1204771859</v>
       </c>
       <c r="J20" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*I20/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.0002875801693</v>
       </c>
       <c r="K20" s="27">
         <f>J20*D20*$B$11</f>
-        <v/>
+        <v>69.85897472</v>
       </c>
       <c r="L20" s="16">
         <f>N20*$B$6/(0.85*$B$5*D20)</f>
-        <v/>
-      </c>
-      <c r="M20" s="17">
+        <v>3.349080882</v>
+      </c>
+      <c r="M20" s="17" t="str">
         <f>IF(L20&lt;=$B$9,"Si (T)","revisar")</f>
-        <v/>
+        <v>Si (T)</v>
       </c>
       <c r="N20" s="27">
         <f>MAX(K20,$B$13)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="O20" s="29">
         <f>ROUNDUP(N20/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="P20" s="22">
         <f>F20*1000000/(0.9*$B$7*$B$11^2)</f>
-        <v/>
+        <v>0.8995629881</v>
       </c>
       <c r="Q20" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*P20/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.002183899739</v>
       </c>
       <c r="R20" s="27">
         <f>Q20*$B$7*$B$11</f>
-        <v/>
+        <v>99.47117335</v>
       </c>
       <c r="S20" s="27">
         <f>MAX(R20,$B$13)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="T20" s="29">
         <f>ROUNDUP(S20/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="U20" s="16">
         <f>0.17*SQRT($B$5)*$B$7*$B$11/1000</f>
-        <v/>
+        <v>40.97250167</v>
       </c>
       <c r="V20" s="16">
         <f>0.75*1.1*U20</f>
-        <v/>
-      </c>
-      <c r="W20" s="17">
+        <v>33.80231387</v>
+      </c>
+      <c r="W20" s="17" t="str">
         <f>IF(H20&lt;=V20,"No requiere","Requiere")</f>
-        <v/>
-      </c>
-      <c r="X20" s="17">
+        <v>No requiere</v>
+      </c>
+      <c r="X20" s="17" t="str">
         <f>IF($B$8&gt;=C20/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="21">
@@ -2785,91 +2785,91 @@
       </c>
       <c r="C21" s="23">
         <f>B21-$B$15</f>
-        <v/>
+        <v>4.45</v>
       </c>
       <c r="D21" s="27">
         <f>MIN(C21*1000/4,$B$7+16*$B$9,$B$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="E21" s="23">
         <f>$B$14*$B$10</f>
-        <v/>
+        <v>10.60096</v>
       </c>
       <c r="F21" s="16">
         <f>E21*C21^2/10</f>
-        <v/>
+        <v>20.99255104</v>
       </c>
       <c r="G21" s="16">
         <f>E21*C21^2/14</f>
-        <v/>
+        <v>14.99467931</v>
       </c>
       <c r="H21" s="16">
         <f>1.15*E21*C21/2</f>
-        <v/>
+        <v>27.1252064</v>
       </c>
       <c r="I21" s="22">
         <f>G21*1000000/(0.9*D21*$B$11^2)</f>
-        <v/>
+        <v>0.2258697727</v>
       </c>
       <c r="J21" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*I21/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.0005403615608</v>
       </c>
       <c r="K21" s="27">
         <f>J21*D21*$B$11</f>
-        <v/>
+        <v>131.2646304</v>
       </c>
       <c r="L21" s="16">
         <f>N21*$B$6/(0.85*$B$5*D21)</f>
-        <v/>
-      </c>
-      <c r="M21" s="17">
+        <v>3.349080882</v>
+      </c>
+      <c r="M21" s="17" t="str">
         <f>IF(L21&lt;=$B$9,"Si (T)","revisar")</f>
-        <v/>
+        <v>Si (T)</v>
       </c>
       <c r="N21" s="27">
         <f>MAX(K21,$B$13)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="O21" s="29">
         <f>ROUNDUP(N21/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="P21" s="22">
         <f>F21*1000000/(0.9*$B$7*$B$11^2)</f>
-        <v/>
+        <v>1.686494303</v>
       </c>
       <c r="Q21" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*P21/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.004168806263</v>
       </c>
       <c r="R21" s="27">
         <f>Q21*$B$7*$B$11</f>
-        <v/>
+        <v>189.8787033</v>
       </c>
       <c r="S21" s="27">
         <f>MAX(R21,$B$13)</f>
-        <v/>
+        <v>189.8787033</v>
       </c>
       <c r="T21" s="29">
         <f>ROUNDUP(S21/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="U21" s="16">
         <f>0.17*SQRT($B$5)*$B$7*$B$11/1000</f>
-        <v/>
+        <v>40.97250167</v>
       </c>
       <c r="V21" s="16">
         <f>0.75*1.1*U21</f>
-        <v/>
-      </c>
-      <c r="W21" s="17">
+        <v>33.80231387</v>
+      </c>
+      <c r="W21" s="17" t="str">
         <f>IF(H21&lt;=V21,"No requiere","Requiere")</f>
-        <v/>
-      </c>
-      <c r="X21" s="17">
+        <v>No requiere</v>
+      </c>
+      <c r="X21" s="17" t="str">
         <f>IF($B$8&gt;=C21/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="22">
@@ -2883,91 +2883,91 @@
       </c>
       <c r="C22" s="23">
         <f>B22-$B$15</f>
-        <v/>
+        <v>4.8</v>
       </c>
       <c r="D22" s="27">
         <f>MIN(C22*1000/4,$B$7+16*$B$9,$B$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="E22" s="23">
         <f>$B$14*$B$10</f>
-        <v/>
+        <v>10.60096</v>
       </c>
       <c r="F22" s="16">
         <f>E22*C22^2/10</f>
-        <v/>
+        <v>24.42461184</v>
       </c>
       <c r="G22" s="16">
         <f>E22*C22^2/14</f>
-        <v/>
+        <v>17.44615131</v>
       </c>
       <c r="H22" s="16">
         <f>1.15*E22*C22/2</f>
-        <v/>
+        <v>29.2586496</v>
       </c>
       <c r="I22" s="22">
         <f>G22*1000000/(0.9*D22*$B$11^2)</f>
-        <v/>
+        <v>0.2627970995</v>
       </c>
       <c r="J22" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*I22/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.0006292005562</v>
       </c>
       <c r="K22" s="27">
         <f>J22*D22*$B$11</f>
-        <v/>
+        <v>152.8453991</v>
       </c>
       <c r="L22" s="16">
         <f>N22*$B$6/(0.85*$B$5*D22)</f>
-        <v/>
-      </c>
-      <c r="M22" s="17">
+        <v>3.371589686</v>
+      </c>
+      <c r="M22" s="17" t="str">
         <f>IF(L22&lt;=$B$9,"Si (T)","revisar")</f>
-        <v/>
+        <v>Si (T)</v>
       </c>
       <c r="N22" s="27">
         <f>MAX(K22,$B$13)</f>
-        <v/>
+        <v>152.8453991</v>
       </c>
       <c r="O22" s="29">
         <f>ROUNDUP(N22/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="P22" s="22">
         <f>F22*1000000/(0.9*$B$7*$B$11^2)</f>
-        <v/>
+        <v>1.962218343</v>
       </c>
       <c r="Q22" s="28">
         <f>(0.85*$B$5/$B$6)*(1-SQRT(1-2*P22/(0.85*$B$5)))</f>
-        <v/>
+        <v>0.004882271123</v>
       </c>
       <c r="R22" s="27">
         <f>Q22*$B$7*$B$11</f>
-        <v/>
+        <v>222.375244</v>
       </c>
       <c r="S22" s="27">
         <f>MAX(R22,$B$13)</f>
-        <v/>
+        <v>222.375244</v>
       </c>
       <c r="T22" s="29">
         <f>ROUNDUP(S22/$B$12,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="U22" s="16">
         <f>0.17*SQRT($B$5)*$B$7*$B$11/1000</f>
-        <v/>
+        <v>40.97250167</v>
       </c>
       <c r="V22" s="16">
         <f>0.75*1.1*U22</f>
-        <v/>
-      </c>
-      <c r="W22" s="17">
+        <v>33.80231387</v>
+      </c>
+      <c r="W22" s="17" t="str">
         <f>IF(H22&lt;=V22,"No requiere","Requiere")</f>
-        <v/>
-      </c>
-      <c r="X22" s="17">
+        <v>No requiere</v>
+      </c>
+      <c r="X22" s="17" t="str">
         <f>IF($B$8&gt;=C22/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="24">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="B5" s="31">
         <f>'Geometria y Verificaciones'!B9*1000</f>
-        <v/>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="B7" s="31">
         <f>B4*B6*B5</f>
-        <v/>
+        <v>108</v>
       </c>
     </row>
     <row r="8">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="B8" s="31">
         <f>MIN(5*B5,450)</f>
-        <v/>
+        <v>300</v>
       </c>
     </row>
     <row r="9">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="B10" s="13">
         <f>3.1416*B9^2/4</f>
-        <v/>
+        <v>28.2744</v>
       </c>
     </row>
     <row r="11">
@@ -3101,7 +3101,7 @@
       </c>
       <c r="B11" s="31">
         <f>B10*1000/B7</f>
-        <v/>
+        <v>261.8</v>
       </c>
     </row>
     <row r="12">
@@ -3120,9 +3120,9 @@
           <t>Estado</t>
         </is>
       </c>
-      <c r="B13" s="34">
+      <c r="B13" s="34" t="str">
         <f>IF(AND(B12&lt;=B8,B12&lt;=B11),"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="15">
@@ -3200,107 +3200,107 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="35">
+      <c r="A5" s="35" t="str">
         <f>Predimensionamiento!A7</f>
-        <v/>
+        <v>T-1</v>
       </c>
       <c r="B5" s="23">
         <f>Predimensionamiento!B7-'Nervios Entrepiso'!$B$15</f>
-        <v/>
+        <v>1.85</v>
       </c>
       <c r="C5" s="16">
         <f>Predimensionamiento!D7</f>
-        <v/>
+        <v>18.5</v>
       </c>
       <c r="D5" s="22">
         <f>B5/C5</f>
-        <v/>
+        <v>0.1</v>
       </c>
       <c r="E5" s="23">
         <f>'Geometria y Verificaciones'!$B$8</f>
-        <v/>
-      </c>
-      <c r="F5" s="17">
+        <v>0.34</v>
+      </c>
+      <c r="F5" s="17" t="str">
         <f>IF(E5&gt;=D5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="35">
+      <c r="A6" s="35" t="str">
         <f>Predimensionamiento!A8</f>
-        <v/>
+        <v>T-2</v>
       </c>
       <c r="B6" s="23">
         <f>Predimensionamiento!B8-'Nervios Entrepiso'!$B$15</f>
-        <v/>
+        <v>3.25</v>
       </c>
       <c r="C6" s="16">
         <f>Predimensionamiento!D8</f>
-        <v/>
+        <v>18.5</v>
       </c>
       <c r="D6" s="22">
         <f>B6/C6</f>
-        <v/>
+        <v>0.1756756757</v>
       </c>
       <c r="E6" s="23">
         <f>'Geometria y Verificaciones'!$B$8</f>
-        <v/>
-      </c>
-      <c r="F6" s="17">
+        <v>0.34</v>
+      </c>
+      <c r="F6" s="17" t="str">
         <f>IF(E6&gt;=D6,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="35">
+      <c r="A7" s="35" t="str">
         <f>Predimensionamiento!A9</f>
-        <v/>
+        <v>T-3</v>
       </c>
       <c r="B7" s="23">
         <f>Predimensionamiento!B9-'Nervios Entrepiso'!$B$15</f>
-        <v/>
+        <v>4.45</v>
       </c>
       <c r="C7" s="16">
         <f>Predimensionamiento!D9</f>
-        <v/>
+        <v>18.5</v>
       </c>
       <c r="D7" s="22">
         <f>B7/C7</f>
-        <v/>
+        <v>0.2405405405</v>
       </c>
       <c r="E7" s="23">
         <f>'Geometria y Verificaciones'!$B$8</f>
-        <v/>
-      </c>
-      <c r="F7" s="17">
+        <v>0.34</v>
+      </c>
+      <c r="F7" s="17" t="str">
         <f>IF(E7&gt;=D7,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="35">
+      <c r="A8" s="35" t="str">
         <f>Predimensionamiento!A10</f>
-        <v/>
+        <v>T-4</v>
       </c>
       <c r="B8" s="23">
         <f>Predimensionamiento!B10-'Nervios Entrepiso'!$B$15</f>
-        <v/>
+        <v>4.8</v>
       </c>
       <c r="C8" s="16">
         <f>Predimensionamiento!D10</f>
-        <v/>
+        <v>18.5</v>
       </c>
       <c r="D8" s="22">
         <f>B8/C8</f>
-        <v/>
+        <v>0.2594594595</v>
       </c>
       <c r="E8" s="23">
         <f>'Geometria y Verificaciones'!$B$8</f>
-        <v/>
-      </c>
-      <c r="F8" s="17">
+        <v>0.34</v>
+      </c>
+      <c r="F8" s="17" t="str">
         <f>IF(E8&gt;=D8,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
     <row r="10">

</xml_diff>